<commit_message>
Normalize four attendee surname capitalizations in Bogotá test workbook
</commit_message>
<xml_diff>
--- a/gs/departuresbogota.xlsx
+++ b/gs/departuresbogota.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attendees" sheetId="1" r:id="Rce421949f0014c6f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Departure Schedule" sheetId="2" r:id="R5c11212061b642ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attendees" sheetId="1" r:id="Rbf4f1a65e4294358"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Departure Schedule" sheetId="2" r:id="R4ad33c1c5d1443e5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -218,9 +218,6 @@
     <x:t xml:space="preserve">Dillon Hylton</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Eddy-Michel CARPIN</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">FAGU</x:t>
   </x:si>
   <x:si>
@@ -242,9 +239,6 @@
     <x:t xml:space="preserve">Jacques Bibrac</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Jonathan CAPRICORNE</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Juan Jose Moran</x:t>
   </x:si>
   <x:si>
@@ -419,9 +413,6 @@
     <x:t xml:space="preserve">AV 092</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Shurman KOOK</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">DUCU</x:t>
   </x:si>
   <x:si>
@@ -561,9 +552,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Silas Martinez</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Widgiz PIERRE</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">David Celis Aguilar</x:t>
@@ -1877,14 +1865,14 @@
       <x:c r="C29" s="4" t="s">
         <x:v>61</x:v>
       </x:c>
-      <x:c r="D29" s="1" t="s">
+      <x:c r="D29" s="1" t="str">
+        <x:v>Eddy-Michel Carpin</x:v>
+      </x:c>
+      <x:c r="E29" s="1">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F29" s="1" t="s">
         <x:v>69</x:v>
-      </x:c>
-      <x:c r="E29" s="1">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F29" s="1" t="s">
-        <x:v>70</x:v>
       </x:c>
       <x:c r="G29" s="1" t="s">
         <x:v>58</x:v>
@@ -1901,7 +1889,7 @@
         <x:v>56</x:v>
       </x:c>
       <x:c r="D30" s="8" t="s">
-        <x:v>71</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="E30" s="8">
         <x:v>1</x:v>
@@ -1924,7 +1912,7 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="D31" s="1" t="s">
-        <x:v>72</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="E31" s="1">
         <x:v>2</x:v>
@@ -1947,7 +1935,7 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="D32" s="8" t="s">
-        <x:v>73</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="E32" s="8">
         <x:v>2</x:v>
@@ -1970,7 +1958,7 @@
         <x:v>56</x:v>
       </x:c>
       <x:c r="D33" s="1" t="s">
-        <x:v>74</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="E33" s="1">
         <x:v>2</x:v>
@@ -1990,16 +1978,16 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="C34" s="9" t="s">
+        <x:v>74</x:v>
+      </x:c>
+      <x:c r="D34" s="8" t="s">
         <x:v>75</x:v>
       </x:c>
-      <x:c r="D34" s="8" t="s">
-        <x:v>76</x:v>
-      </x:c>
       <x:c r="E34" s="8">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F34" s="8" t="s">
-        <x:v>70</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="G34" s="8" t="s">
         <x:v>58</x:v>
@@ -2015,14 +2003,14 @@
       <x:c r="C35" s="4" t="s">
         <x:v>56</x:v>
       </x:c>
-      <x:c r="D35" s="1" t="s">
-        <x:v>77</x:v>
+      <x:c r="D35" s="1" t="str">
+        <x:v>Jonathan Capricorne</x:v>
       </x:c>
       <x:c r="E35" s="1">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F35" s="1" t="s">
-        <x:v>70</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="G35" s="1" t="s">
         <x:v>58</x:v>
@@ -2039,7 +2027,7 @@
         <x:v>56</x:v>
       </x:c>
       <x:c r="D36" s="8" t="s">
-        <x:v>78</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="E36" s="8">
         <x:v>1</x:v>
@@ -2062,7 +2050,7 @@
         <x:v>56</x:v>
       </x:c>
       <x:c r="D37" s="1" t="s">
-        <x:v>79</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="E37" s="1">
         <x:v>2</x:v>
@@ -2085,7 +2073,7 @@
         <x:v>56</x:v>
       </x:c>
       <x:c r="D38" s="8" t="s">
-        <x:v>80</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="E38" s="8">
         <x:v>1</x:v>
@@ -2108,7 +2096,7 @@
         <x:v>56</x:v>
       </x:c>
       <x:c r="D39" s="1" t="s">
-        <x:v>81</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="E39" s="1">
         <x:v>1</x:v>
@@ -2131,7 +2119,7 @@
         <x:v>56</x:v>
       </x:c>
       <x:c r="D40" s="8" t="s">
-        <x:v>82</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="E40" s="8">
         <x:v>1</x:v>
@@ -2154,13 +2142,13 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="D41" s="1" t="s">
-        <x:v>83</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="E41" s="1">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F41" s="1" t="s">
-        <x:v>70</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="G41" s="1" t="s">
         <x:v>58</x:v>
@@ -2177,7 +2165,7 @@
         <x:v>56</x:v>
       </x:c>
       <x:c r="D42" s="8" t="s">
-        <x:v>84</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="E42" s="8">
         <x:v>2</x:v>
@@ -2194,22 +2182,22 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B43" s="1" t="s">
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="C43" s="4" t="s">
+        <x:v>84</x:v>
+      </x:c>
+      <x:c r="D43" s="1" t="s">
         <x:v>85</x:v>
       </x:c>
-      <x:c r="C43" s="4" t="s">
+      <x:c r="E43" s="1">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F43" s="1" t="s">
         <x:v>86</x:v>
       </x:c>
-      <x:c r="D43" s="1" t="s">
+      <x:c r="G43" s="1" t="s">
         <x:v>87</x:v>
-      </x:c>
-      <x:c r="E43" s="1">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F43" s="1" t="s">
-        <x:v>88</x:v>
-      </x:c>
-      <x:c r="G43" s="1" t="s">
-        <x:v>89</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
@@ -2217,22 +2205,22 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B44" s="8" t="s">
-        <x:v>85</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="C44" s="9" t="s">
+        <x:v>84</x:v>
+      </x:c>
+      <x:c r="D44" s="8" t="s">
+        <x:v>88</x:v>
+      </x:c>
+      <x:c r="E44" s="8">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F44" s="8" t="s">
         <x:v>86</x:v>
       </x:c>
-      <x:c r="D44" s="8" t="s">
-        <x:v>90</x:v>
-      </x:c>
-      <x:c r="E44" s="8">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F44" s="8" t="s">
-        <x:v>88</x:v>
-      </x:c>
       <x:c r="G44" s="8" t="s">
-        <x:v>89</x:v>
+        <x:v>87</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
@@ -2240,13 +2228,13 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B45" s="1" t="s">
-        <x:v>85</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="C45" s="4" t="s">
-        <x:v>91</x:v>
+        <x:v>89</x:v>
       </x:c>
       <x:c r="D45" s="1" t="s">
-        <x:v>92</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="E45" s="1">
         <x:v>1</x:v>
@@ -2255,7 +2243,7 @@
         <x:v>45</x:v>
       </x:c>
       <x:c r="G45" s="1" t="s">
-        <x:v>89</x:v>
+        <x:v>87</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
@@ -2263,22 +2251,22 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B46" s="8" t="s">
-        <x:v>85</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="C46" s="9" t="s">
-        <x:v>93</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="D46" s="8" t="s">
-        <x:v>94</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="E46" s="8">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F46" s="8" t="s">
-        <x:v>88</x:v>
+        <x:v>86</x:v>
       </x:c>
       <x:c r="G46" s="8" t="s">
-        <x:v>89</x:v>
+        <x:v>87</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
@@ -2286,19 +2274,19 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B47" s="1" t="s">
-        <x:v>85</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="C47" s="4" t="s">
+        <x:v>93</x:v>
+      </x:c>
+      <x:c r="D47" s="1" t="s">
+        <x:v>94</x:v>
+      </x:c>
+      <x:c r="E47" s="1">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F47" s="1" t="s">
         <x:v>95</x:v>
-      </x:c>
-      <x:c r="D47" s="1" t="s">
-        <x:v>96</x:v>
-      </x:c>
-      <x:c r="E47" s="1">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F47" s="1" t="s">
-        <x:v>97</x:v>
       </x:c>
       <x:c r="G47" s="1" t="s">
         <x:v>50</x:v>
@@ -2309,13 +2297,13 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B48" s="8" t="s">
-        <x:v>85</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="C48" s="9" t="s">
-        <x:v>98</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="D48" s="8" t="s">
-        <x:v>99</x:v>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="E48" s="8">
         <x:v>1</x:v>
@@ -2324,7 +2312,7 @@
         <x:v>54</x:v>
       </x:c>
       <x:c r="G48" s="8" t="s">
-        <x:v>89</x:v>
+        <x:v>87</x:v>
       </x:c>
     </x:row>
     <x:row r="49">
@@ -2332,22 +2320,22 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B49" s="1" t="s">
-        <x:v>85</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="C49" s="4" t="s">
-        <x:v>93</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="D49" s="1" t="s">
-        <x:v>100</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="E49" s="1">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F49" s="1" t="s">
-        <x:v>101</x:v>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="G49" s="1" t="s">
-        <x:v>89</x:v>
+        <x:v>87</x:v>
       </x:c>
     </x:row>
     <x:row r="50">
@@ -2355,22 +2343,22 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B50" s="8" t="s">
-        <x:v>85</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="C50" s="9" t="s">
-        <x:v>93</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="D50" s="8" t="s">
-        <x:v>102</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="E50" s="8">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F50" s="8" t="s">
-        <x:v>97</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="G50" s="8" t="s">
-        <x:v>89</x:v>
+        <x:v>87</x:v>
       </x:c>
     </x:row>
     <x:row r="51">
@@ -2378,22 +2366,22 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B51" s="1" t="s">
-        <x:v>85</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="C51" s="4" t="s">
-        <x:v>93</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="D51" s="1" t="s">
-        <x:v>103</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="E51" s="1">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F51" s="1" t="s">
-        <x:v>101</x:v>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="G51" s="1" t="s">
-        <x:v>89</x:v>
+        <x:v>87</x:v>
       </x:c>
     </x:row>
     <x:row r="52">
@@ -2401,13 +2389,13 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B52" s="8" t="s">
-        <x:v>85</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="C52" s="9" t="s">
-        <x:v>86</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="D52" s="8" t="s">
-        <x:v>104</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="E52" s="8">
         <x:v>1</x:v>
@@ -2416,7 +2404,7 @@
         <x:v>54</x:v>
       </x:c>
       <x:c r="G52" s="8" t="s">
-        <x:v>89</x:v>
+        <x:v>87</x:v>
       </x:c>
     </x:row>
     <x:row r="53">
@@ -2424,13 +2412,13 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B53" s="1" t="s">
-        <x:v>85</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="C53" s="4" t="s">
-        <x:v>93</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="D53" s="1" t="s">
-        <x:v>105</x:v>
+        <x:v>103</x:v>
       </x:c>
       <x:c r="E53" s="1">
         <x:v>1</x:v>
@@ -2439,7 +2427,7 @@
         <x:v>45</x:v>
       </x:c>
       <x:c r="G53" s="1" t="s">
-        <x:v>89</x:v>
+        <x:v>87</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
@@ -2447,19 +2435,19 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B54" s="8" t="s">
-        <x:v>85</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="C54" s="9" t="s">
-        <x:v>106</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="D54" s="8" t="s">
-        <x:v>107</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="E54" s="8">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F54" s="8" t="s">
-        <x:v>97</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="G54" s="8" t="s">
         <x:v>50</x:v>
@@ -2470,22 +2458,22 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B55" s="1" t="s">
-        <x:v>85</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="C55" s="4" t="s">
-        <x:v>86</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="D55" s="1" t="s">
-        <x:v>108</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="E55" s="1">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F55" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="G55" s="1" t="s">
-        <x:v>89</x:v>
+        <x:v>87</x:v>
       </x:c>
     </x:row>
     <x:row r="56">
@@ -2493,13 +2481,13 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B56" s="8" t="s">
-        <x:v>85</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="C56" s="9" t="s">
-        <x:v>86</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="D56" s="8" t="s">
-        <x:v>110</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="E56" s="8">
         <x:v>1</x:v>
@@ -2508,7 +2496,7 @@
         <x:v>54</x:v>
       </x:c>
       <x:c r="G56" s="8" t="s">
-        <x:v>89</x:v>
+        <x:v>87</x:v>
       </x:c>
     </x:row>
     <x:row r="57">
@@ -2516,22 +2504,22 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B57" s="1" t="s">
-        <x:v>85</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="C57" s="4" t="s">
-        <x:v>86</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="D57" s="1" t="s">
-        <x:v>111</x:v>
+        <x:v>109</x:v>
       </x:c>
       <x:c r="E57" s="1">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F57" s="1" t="s">
-        <x:v>101</x:v>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="G57" s="1" t="s">
-        <x:v>89</x:v>
+        <x:v>87</x:v>
       </x:c>
     </x:row>
     <x:row r="58">
@@ -2539,22 +2527,22 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B58" s="8" t="s">
-        <x:v>85</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="C58" s="9" t="s">
+        <x:v>110</x:v>
+      </x:c>
+      <x:c r="D58" s="8" t="s">
+        <x:v>111</x:v>
+      </x:c>
+      <x:c r="E58" s="8">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F58" s="8" t="s">
         <x:v>112</x:v>
       </x:c>
-      <x:c r="D58" s="8" t="s">
-        <x:v>113</x:v>
-      </x:c>
-      <x:c r="E58" s="8">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F58" s="8" t="s">
-        <x:v>114</x:v>
-      </x:c>
       <x:c r="G58" s="8" t="s">
-        <x:v>89</x:v>
+        <x:v>87</x:v>
       </x:c>
     </x:row>
     <x:row r="59">
@@ -2568,7 +2556,7 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="D59" s="1" t="s">
-        <x:v>115</x:v>
+        <x:v>113</x:v>
       </x:c>
       <x:c r="E59" s="1">
         <x:v>1</x:v>
@@ -2585,22 +2573,22 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B60" s="8" t="s">
-        <x:v>85</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="C60" s="9" t="s">
-        <x:v>93</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="D60" s="8" t="s">
-        <x:v>116</x:v>
+        <x:v>114</x:v>
       </x:c>
       <x:c r="E60" s="8">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F60" s="8" t="s">
-        <x:v>101</x:v>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="G60" s="8" t="s">
-        <x:v>89</x:v>
+        <x:v>87</x:v>
       </x:c>
     </x:row>
     <x:row r="61">
@@ -2608,19 +2596,19 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B61" s="1" t="s">
-        <x:v>85</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="C61" s="4" t="s">
-        <x:v>117</x:v>
+        <x:v>115</x:v>
       </x:c>
       <x:c r="D61" s="1" t="s">
-        <x:v>118</x:v>
+        <x:v>116</x:v>
       </x:c>
       <x:c r="E61" s="1">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F61" s="1" t="s">
-        <x:v>97</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="G61" s="1" t="s">
         <x:v>50</x:v>
@@ -2631,22 +2619,22 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B62" s="8" t="s">
-        <x:v>85</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="C62" s="9" t="s">
-        <x:v>93</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="D62" s="8" t="s">
-        <x:v>119</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="E62" s="8">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F62" s="8" t="s">
-        <x:v>88</x:v>
+        <x:v>86</x:v>
       </x:c>
       <x:c r="G62" s="8" t="s">
-        <x:v>89</x:v>
+        <x:v>87</x:v>
       </x:c>
     </x:row>
     <x:row r="63">
@@ -2654,22 +2642,22 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B63" s="1" t="s">
-        <x:v>85</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="C63" s="4" t="s">
-        <x:v>93</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="D63" s="1" t="s">
-        <x:v>120</x:v>
+        <x:v>118</x:v>
       </x:c>
       <x:c r="E63" s="1">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F63" s="1" t="s">
-        <x:v>101</x:v>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="G63" s="1" t="s">
-        <x:v>89</x:v>
+        <x:v>87</x:v>
       </x:c>
     </x:row>
     <x:row r="64">
@@ -2677,19 +2665,19 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B64" s="8" t="s">
+        <x:v>119</x:v>
+      </x:c>
+      <x:c r="C64" s="9" t="s">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="D64" s="8" t="s">
         <x:v>121</x:v>
       </x:c>
-      <x:c r="C64" s="9" t="s">
+      <x:c r="E64" s="8">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F64" s="8" t="s">
         <x:v>122</x:v>
-      </x:c>
-      <x:c r="D64" s="8" t="s">
-        <x:v>123</x:v>
-      </x:c>
-      <x:c r="E64" s="8">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F64" s="8" t="s">
-        <x:v>124</x:v>
       </x:c>
       <x:c r="G64" s="8" t="s">
         <x:v>50</x:v>
@@ -2700,19 +2688,19 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B65" s="1" t="s">
-        <x:v>121</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="C65" s="4" t="s">
-        <x:v>125</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="D65" s="1" t="s">
-        <x:v>126</x:v>
+        <x:v>124</x:v>
       </x:c>
       <x:c r="E65" s="1">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F65" s="1" t="s">
-        <x:v>124</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="G65" s="1" t="s">
         <x:v>50</x:v>
@@ -2723,19 +2711,19 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B66" s="8" t="s">
-        <x:v>121</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="C66" s="9" t="s">
+        <x:v>123</x:v>
+      </x:c>
+      <x:c r="D66" s="8" t="s">
         <x:v>125</x:v>
       </x:c>
-      <x:c r="D66" s="8" t="s">
-        <x:v>127</x:v>
-      </x:c>
       <x:c r="E66" s="8">
         <x:v>2</x:v>
       </x:c>
       <x:c r="F66" s="8" t="s">
-        <x:v>124</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="G66" s="8" t="s">
         <x:v>50</x:v>
@@ -2746,19 +2734,19 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B67" s="1" t="s">
-        <x:v>121</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="C67" s="4" t="s">
-        <x:v>125</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="D67" s="1" t="s">
-        <x:v>128</x:v>
+        <x:v>126</x:v>
       </x:c>
       <x:c r="E67" s="1">
         <x:v>2</x:v>
       </x:c>
       <x:c r="F67" s="1" t="s">
-        <x:v>124</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="G67" s="1" t="s">
         <x:v>50</x:v>
@@ -2769,22 +2757,22 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B68" s="8" t="s">
+        <x:v>127</x:v>
+      </x:c>
+      <x:c r="C68" s="9" t="s">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="D68" s="8" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="C68" s="9" t="s">
+      <x:c r="E68" s="8">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F68" s="8" t="s">
         <x:v>130</x:v>
       </x:c>
-      <x:c r="D68" s="8" t="s">
+      <x:c r="G68" s="8" t="s">
         <x:v>131</x:v>
-      </x:c>
-      <x:c r="E68" s="8">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F68" s="8" t="s">
-        <x:v>132</x:v>
-      </x:c>
-      <x:c r="G68" s="8" t="s">
-        <x:v>133</x:v>
       </x:c>
     </x:row>
     <x:row r="69">
@@ -2792,19 +2780,19 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B69" s="1" t="s">
+        <x:v>132</x:v>
+      </x:c>
+      <x:c r="C69" s="4" t="s">
+        <x:v>133</x:v>
+      </x:c>
+      <x:c r="D69" s="1" t="str">
+        <x:v>Shurman Kook</x:v>
+      </x:c>
+      <x:c r="E69" s="1">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F69" s="1" t="s">
         <x:v>134</x:v>
-      </x:c>
-      <x:c r="C69" s="4" t="s">
-        <x:v>135</x:v>
-      </x:c>
-      <x:c r="D69" s="1" t="s">
-        <x:v>136</x:v>
-      </x:c>
-      <x:c r="E69" s="1">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F69" s="1" t="s">
-        <x:v>137</x:v>
       </x:c>
       <x:c r="G69" s="1" t="s">
         <x:v>50</x:v>
@@ -2815,19 +2803,19 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B70" s="8" t="s">
+        <x:v>135</x:v>
+      </x:c>
+      <x:c r="C70" s="9" t="s">
+        <x:v>136</x:v>
+      </x:c>
+      <x:c r="D70" s="8" t="s">
+        <x:v>137</x:v>
+      </x:c>
+      <x:c r="E70" s="8">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F70" s="8" t="s">
         <x:v>138</x:v>
-      </x:c>
-      <x:c r="C70" s="9" t="s">
-        <x:v>139</x:v>
-      </x:c>
-      <x:c r="D70" s="8" t="s">
-        <x:v>140</x:v>
-      </x:c>
-      <x:c r="E70" s="8">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F70" s="8" t="s">
-        <x:v>141</x:v>
       </x:c>
       <x:c r="G70" s="8" t="s">
         <x:v>14</x:v>
@@ -2838,19 +2826,19 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B71" s="1" t="s">
-        <x:v>138</x:v>
+        <x:v>135</x:v>
       </x:c>
       <x:c r="C71" s="4" t="s">
+        <x:v>136</x:v>
+      </x:c>
+      <x:c r="D71" s="1" t="s">
         <x:v>139</x:v>
       </x:c>
-      <x:c r="D71" s="1" t="s">
-        <x:v>142</x:v>
-      </x:c>
       <x:c r="E71" s="1">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F71" s="1" t="s">
-        <x:v>143</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="G71" s="1" t="s">
         <x:v>14</x:v>
@@ -2861,19 +2849,19 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B72" s="8" t="s">
-        <x:v>138</x:v>
+        <x:v>135</x:v>
       </x:c>
       <x:c r="C72" s="9" t="s">
-        <x:v>139</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="D72" s="8" t="s">
-        <x:v>144</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="E72" s="8">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F72" s="8" t="s">
-        <x:v>145</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="G72" s="8" t="s">
         <x:v>14</x:v>
@@ -2884,19 +2872,19 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B73" s="1" t="s">
+        <x:v>135</x:v>
+      </x:c>
+      <x:c r="C73" s="1" t="s">
+        <x:v>136</x:v>
+      </x:c>
+      <x:c r="D73" s="1" t="s">
+        <x:v>143</x:v>
+      </x:c>
+      <x:c r="E73" s="1">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F73" s="1" t="s">
         <x:v>138</x:v>
-      </x:c>
-      <x:c r="C73" s="1" t="s">
-        <x:v>139</x:v>
-      </x:c>
-      <x:c r="D73" s="1" t="s">
-        <x:v>146</x:v>
-      </x:c>
-      <x:c r="E73" s="1">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F73" s="1" t="s">
-        <x:v>141</x:v>
       </x:c>
       <x:c r="G73" s="1" t="s">
         <x:v>14</x:v>
@@ -2907,19 +2895,19 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B74" s="8" t="s">
-        <x:v>138</x:v>
+        <x:v>135</x:v>
       </x:c>
       <x:c r="C74" s="9" t="s">
-        <x:v>139</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="D74" s="8" t="s">
-        <x:v>147</x:v>
+        <x:v>144</x:v>
       </x:c>
       <x:c r="E74" s="8">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F74" s="8" t="s">
-        <x:v>145</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="G74" s="8" t="s">
         <x:v>14</x:v>
@@ -2930,19 +2918,19 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B75" s="1" t="s">
-        <x:v>138</x:v>
+        <x:v>135</x:v>
       </x:c>
       <x:c r="C75" s="4" t="s">
-        <x:v>139</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="D75" s="1" t="s">
-        <x:v>148</x:v>
+        <x:v>145</x:v>
       </x:c>
       <x:c r="E75" s="1">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F75" s="1" t="s">
-        <x:v>143</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="G75" s="1" t="s">
         <x:v>14</x:v>
@@ -2953,19 +2941,19 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B76" s="8" t="s">
+        <x:v>135</x:v>
+      </x:c>
+      <x:c r="C76" s="9" t="s">
+        <x:v>146</x:v>
+      </x:c>
+      <x:c r="D76" s="8" t="s">
+        <x:v>147</x:v>
+      </x:c>
+      <x:c r="E76" s="8">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F76" s="8" t="s">
         <x:v>138</x:v>
-      </x:c>
-      <x:c r="C76" s="9" t="s">
-        <x:v>149</x:v>
-      </x:c>
-      <x:c r="D76" s="8" t="s">
-        <x:v>150</x:v>
-      </x:c>
-      <x:c r="E76" s="8">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F76" s="8" t="s">
-        <x:v>141</x:v>
       </x:c>
       <x:c r="G76" s="8" t="s">
         <x:v>14</x:v>
@@ -2976,19 +2964,19 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B77" s="1" t="s">
-        <x:v>138</x:v>
+        <x:v>135</x:v>
       </x:c>
       <x:c r="C77" s="4" t="s">
-        <x:v>151</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="D77" s="1" t="s">
-        <x:v>152</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="E77" s="1">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F77" s="1" t="s">
-        <x:v>143</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="G77" s="1" t="s">
         <x:v>14</x:v>
@@ -2999,13 +2987,13 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B78" s="8" t="s">
-        <x:v>138</x:v>
+        <x:v>135</x:v>
       </x:c>
       <x:c r="C78" s="9" t="s">
-        <x:v>149</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="D78" s="8" t="s">
-        <x:v>153</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="E78" s="8">
         <x:v>2</x:v>
@@ -3022,19 +3010,19 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B79" s="1" t="s">
-        <x:v>138</x:v>
+        <x:v>135</x:v>
       </x:c>
       <x:c r="C79" s="4" t="s">
-        <x:v>139</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="D79" s="1" t="s">
-        <x:v>154</x:v>
+        <x:v>151</x:v>
       </x:c>
       <x:c r="E79" s="1">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F79" s="1" t="s">
-        <x:v>143</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="G79" s="1" t="s">
         <x:v>14</x:v>
@@ -3045,19 +3033,19 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B80" s="8" t="s">
-        <x:v>138</x:v>
+        <x:v>135</x:v>
       </x:c>
       <x:c r="C80" s="9" t="s">
-        <x:v>139</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="D80" s="8" t="s">
-        <x:v>155</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="E80" s="8">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F80" s="8" t="s">
-        <x:v>145</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="G80" s="8" t="s">
         <x:v>14</x:v>
@@ -3068,19 +3056,19 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B81" s="1" t="s">
-        <x:v>138</x:v>
+        <x:v>135</x:v>
       </x:c>
       <x:c r="C81" s="4" t="s">
-        <x:v>139</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="D81" s="1" t="s">
-        <x:v>156</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="E81" s="1">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F81" s="1" t="s">
-        <x:v>145</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="G81" s="1" t="s">
         <x:v>14</x:v>
@@ -3091,19 +3079,19 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B82" s="8" t="s">
-        <x:v>138</x:v>
+        <x:v>135</x:v>
       </x:c>
       <x:c r="C82" s="9" t="s">
-        <x:v>157</x:v>
+        <x:v>154</x:v>
       </x:c>
       <x:c r="D82" s="8" t="s">
-        <x:v>158</x:v>
+        <x:v>155</x:v>
       </x:c>
       <x:c r="E82" s="8">
         <x:v>2</x:v>
       </x:c>
       <x:c r="F82" s="8" t="s">
-        <x:v>145</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="G82" s="8" t="s">
         <x:v>14</x:v>
@@ -3114,22 +3102,22 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B83" s="1" t="s">
+        <x:v>156</x:v>
+      </x:c>
+      <x:c r="C83" s="4" t="s">
+        <x:v>157</x:v>
+      </x:c>
+      <x:c r="D83" s="1" t="s">
+        <x:v>158</x:v>
+      </x:c>
+      <x:c r="E83" s="1">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F83" s="1" t="s">
+        <x:v>130</x:v>
+      </x:c>
+      <x:c r="G83" s="1" t="s">
         <x:v>159</x:v>
-      </x:c>
-      <x:c r="C83" s="4" t="s">
-        <x:v>160</x:v>
-      </x:c>
-      <x:c r="D83" s="1" t="s">
-        <x:v>161</x:v>
-      </x:c>
-      <x:c r="E83" s="1">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F83" s="1" t="s">
-        <x:v>132</x:v>
-      </x:c>
-      <x:c r="G83" s="1" t="s">
-        <x:v>162</x:v>
       </x:c>
     </x:row>
     <x:row r="84">
@@ -3137,22 +3125,22 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B84" s="8" t="s">
+        <x:v>160</x:v>
+      </x:c>
+      <x:c r="C84" s="9" t="s">
+        <x:v>161</x:v>
+      </x:c>
+      <x:c r="D84" s="8" t="s">
+        <x:v>162</x:v>
+      </x:c>
+      <x:c r="E84" s="8">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F84" s="8" t="s">
         <x:v>163</x:v>
       </x:c>
-      <x:c r="C84" s="9" t="s">
+      <x:c r="G84" s="8" t="s">
         <x:v>164</x:v>
-      </x:c>
-      <x:c r="D84" s="8" t="s">
-        <x:v>165</x:v>
-      </x:c>
-      <x:c r="E84" s="8">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F84" s="8" t="s">
-        <x:v>166</x:v>
-      </x:c>
-      <x:c r="G84" s="8" t="s">
-        <x:v>167</x:v>
       </x:c>
     </x:row>
     <x:row r="85">
@@ -3160,19 +3148,19 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B85" s="1" t="s">
-        <x:v>168</x:v>
+        <x:v>165</x:v>
       </x:c>
       <x:c r="C85" s="4" t="s">
-        <x:v>169</x:v>
+        <x:v>166</x:v>
       </x:c>
       <x:c r="D85" s="1" t="s">
-        <x:v>170</x:v>
+        <x:v>167</x:v>
       </x:c>
       <x:c r="E85" s="1">
         <x:v>2</x:v>
       </x:c>
       <x:c r="F85" s="1" t="s">
-        <x:v>143</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="G85" s="1" t="s">
         <x:v>14</x:v>
@@ -3183,13 +3171,13 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B86" s="8" t="s">
-        <x:v>171</x:v>
+        <x:v>168</x:v>
       </x:c>
       <x:c r="C86" s="9" t="s">
-        <x:v>172</x:v>
+        <x:v>169</x:v>
       </x:c>
       <x:c r="D86" s="8" t="s">
-        <x:v>173</x:v>
+        <x:v>170</x:v>
       </x:c>
       <x:c r="E86" s="8">
         <x:v>3</x:v>
@@ -3206,13 +3194,13 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B87" s="1" t="s">
+        <x:v>168</x:v>
+      </x:c>
+      <x:c r="C87" s="4" t="s">
         <x:v>171</x:v>
       </x:c>
-      <x:c r="C87" s="4" t="s">
-        <x:v>174</x:v>
-      </x:c>
       <x:c r="D87" s="1" t="s">
-        <x:v>175</x:v>
+        <x:v>172</x:v>
       </x:c>
       <x:c r="E87" s="1">
         <x:v>2</x:v>
@@ -3229,19 +3217,19 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B88" s="8" t="s">
-        <x:v>171</x:v>
+        <x:v>168</x:v>
       </x:c>
       <x:c r="C88" s="9" t="s">
-        <x:v>176</x:v>
+        <x:v>173</x:v>
       </x:c>
       <x:c r="D88" s="8" t="s">
-        <x:v>177</x:v>
+        <x:v>174</x:v>
       </x:c>
       <x:c r="E88" s="8">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F88" s="8" t="s">
-        <x:v>178</x:v>
+        <x:v>175</x:v>
       </x:c>
       <x:c r="G88" s="8" t="s">
         <x:v>50</x:v>
@@ -3252,13 +3240,13 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B89" s="1" t="s">
-        <x:v>171</x:v>
+        <x:v>168</x:v>
       </x:c>
       <x:c r="C89" s="4" t="s">
-        <x:v>179</x:v>
+        <x:v>176</x:v>
       </x:c>
       <x:c r="D89" s="1" t="s">
-        <x:v>180</x:v>
+        <x:v>177</x:v>
       </x:c>
       <x:c r="E89" s="1">
         <x:v>2</x:v>
@@ -3275,19 +3263,19 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B90" s="8" t="s">
-        <x:v>171</x:v>
+        <x:v>168</x:v>
       </x:c>
       <x:c r="C90" s="9" t="s">
-        <x:v>181</x:v>
+        <x:v>178</x:v>
       </x:c>
       <x:c r="D90" s="8" t="s">
-        <x:v>182</x:v>
+        <x:v>179</x:v>
       </x:c>
       <x:c r="E90" s="8">
         <x:v>2</x:v>
       </x:c>
       <x:c r="F90" s="8" t="s">
-        <x:v>178</x:v>
+        <x:v>175</x:v>
       </x:c>
       <x:c r="G90" s="8" t="s">
         <x:v>14</x:v>
@@ -3298,13 +3286,13 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B91" s="1" t="s">
-        <x:v>171</x:v>
+        <x:v>168</x:v>
       </x:c>
       <x:c r="C91" s="4" t="s">
-        <x:v>172</x:v>
+        <x:v>169</x:v>
       </x:c>
       <x:c r="D91" s="1" t="s">
-        <x:v>183</x:v>
+        <x:v>180</x:v>
       </x:c>
       <x:c r="E91" s="1">
         <x:v>2</x:v>
@@ -3326,14 +3314,14 @@
       <x:c r="C92" s="9" t="s">
         <x:v>56</x:v>
       </x:c>
-      <x:c r="D92" s="8" t="s">
-        <x:v>184</x:v>
+      <x:c r="D92" s="8" t="str">
+        <x:v>Widgiz Pierre</x:v>
       </x:c>
       <x:c r="E92" s="8">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F92" s="8" t="s">
-        <x:v>70</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="G92" s="8" t="s">
         <x:v>58</x:v>
@@ -3347,10 +3335,10 @@
         <x:v>0.33333333333333331</x:v>
       </x:c>
       <x:c r="C93" s="4" t="s">
-        <x:v>86</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="D93" s="1" t="s">
-        <x:v>185</x:v>
+        <x:v>181</x:v>
       </x:c>
       <x:c r="E93" s="1">
         <x:v>1</x:v>
@@ -3359,7 +3347,7 @@
         <x:v>45</x:v>
       </x:c>
       <x:c r="G93" s="1" t="s">
-        <x:v>89</x:v>
+        <x:v>87</x:v>
       </x:c>
     </x:row>
     <x:row r="94">
@@ -3367,19 +3355,19 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B94" s="8" t="s">
-        <x:v>186</x:v>
+        <x:v>182</x:v>
       </x:c>
       <x:c r="C94" s="9" t="s">
-        <x:v>187</x:v>
+        <x:v>183</x:v>
       </x:c>
       <x:c r="D94" s="8" t="s">
-        <x:v>188</x:v>
+        <x:v>184</x:v>
       </x:c>
       <x:c r="E94" s="8">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F94" s="8" t="s">
-        <x:v>141</x:v>
+        <x:v>138</x:v>
       </x:c>
       <x:c r="G94" s="8" t="s">
         <x:v>14</x:v>
@@ -3390,13 +3378,13 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B95" s="1" t="s">
-        <x:v>189</x:v>
+        <x:v>185</x:v>
       </x:c>
       <x:c r="C95" s="4" t="s">
-        <x:v>190</x:v>
+        <x:v>186</x:v>
       </x:c>
       <x:c r="D95" s="1" t="s">
-        <x:v>191</x:v>
+        <x:v>187</x:v>
       </x:c>
       <x:c r="E95" s="1">
         <x:v>2</x:v>
@@ -3413,13 +3401,13 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B96" s="8" t="s">
-        <x:v>189</x:v>
+        <x:v>185</x:v>
       </x:c>
       <x:c r="C96" s="9" t="s">
-        <x:v>190</x:v>
+        <x:v>186</x:v>
       </x:c>
       <x:c r="D96" s="8" t="s">
-        <x:v>192</x:v>
+        <x:v>188</x:v>
       </x:c>
       <x:c r="E96" s="8">
         <x:v>1</x:v>
@@ -3436,19 +3424,19 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B97" s="1" t="s">
-        <x:v>193</x:v>
+        <x:v>189</x:v>
       </x:c>
       <x:c r="C97" s="4" t="s">
-        <x:v>194</x:v>
+        <x:v>190</x:v>
       </x:c>
       <x:c r="D97" s="1" t="s">
-        <x:v>195</x:v>
+        <x:v>191</x:v>
       </x:c>
       <x:c r="E97" s="1">
         <x:v>2</x:v>
       </x:c>
       <x:c r="F97" s="1" t="s">
-        <x:v>141</x:v>
+        <x:v>138</x:v>
       </x:c>
       <x:c r="G97" s="1" t="s">
         <x:v>50</x:v>
@@ -3459,19 +3447,19 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B98" s="8" t="s">
-        <x:v>196</x:v>
+        <x:v>192</x:v>
       </x:c>
       <x:c r="C98" s="9" t="s">
-        <x:v>197</x:v>
+        <x:v>193</x:v>
       </x:c>
       <x:c r="D98" s="8" t="s">
-        <x:v>198</x:v>
+        <x:v>194</x:v>
       </x:c>
       <x:c r="E98" s="8">
         <x:v>2</x:v>
       </x:c>
       <x:c r="F98" s="8" t="s">
-        <x:v>199</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="G98" s="8" t="s">
         <x:v>50</x:v>
@@ -3482,19 +3470,19 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B99" s="1" t="s">
+        <x:v>192</x:v>
+      </x:c>
+      <x:c r="C99" s="4" t="s">
+        <x:v>193</x:v>
+      </x:c>
+      <x:c r="D99" s="1" t="s">
         <x:v>196</x:v>
       </x:c>
-      <x:c r="C99" s="4" t="s">
-        <x:v>197</x:v>
-      </x:c>
-      <x:c r="D99" s="1" t="s">
-        <x:v>200</x:v>
-      </x:c>
       <x:c r="E99" s="1">
         <x:v>2</x:v>
       </x:c>
       <x:c r="F99" s="1" t="s">
-        <x:v>199</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="G99" s="1" t="s">
         <x:v>50</x:v>
@@ -3505,13 +3493,13 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B100" s="8" t="s">
-        <x:v>196</x:v>
+        <x:v>192</x:v>
       </x:c>
       <x:c r="C100" s="9" t="s">
+        <x:v>193</x:v>
+      </x:c>
+      <x:c r="D100" s="8" t="s">
         <x:v>197</x:v>
-      </x:c>
-      <x:c r="D100" s="8" t="s">
-        <x:v>201</x:v>
       </x:c>
       <x:c r="E100" s="8">
         <x:v>1</x:v>
@@ -3528,13 +3516,13 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B101" s="1" t="s">
-        <x:v>196</x:v>
+        <x:v>192</x:v>
       </x:c>
       <x:c r="C101" s="4" t="s">
-        <x:v>202</x:v>
+        <x:v>198</x:v>
       </x:c>
       <x:c r="D101" s="1" t="s">
-        <x:v>203</x:v>
+        <x:v>199</x:v>
       </x:c>
       <x:c r="E101" s="1">
         <x:v>1</x:v>
@@ -3551,19 +3539,19 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B102" s="8" t="s">
-        <x:v>204</x:v>
+        <x:v>200</x:v>
       </x:c>
       <x:c r="C102" s="9" t="s">
-        <x:v>205</x:v>
+        <x:v>201</x:v>
       </x:c>
       <x:c r="D102" s="8" t="s">
-        <x:v>206</x:v>
+        <x:v>202</x:v>
       </x:c>
       <x:c r="E102" s="8">
         <x:v>2</x:v>
       </x:c>
       <x:c r="F102" s="8" t="s">
-        <x:v>137</x:v>
+        <x:v>134</x:v>
       </x:c>
       <x:c r="G102" s="8" t="s">
         <x:v>50</x:v>
@@ -3574,19 +3562,19 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B103" s="1" t="s">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="C103" s="4" t="s">
+        <x:v>203</x:v>
+      </x:c>
+      <x:c r="D103" s="1" t="s">
         <x:v>204</x:v>
       </x:c>
-      <x:c r="C103" s="4" t="s">
-        <x:v>207</x:v>
-      </x:c>
-      <x:c r="D103" s="1" t="s">
-        <x:v>208</x:v>
-      </x:c>
       <x:c r="E103" s="1">
         <x:v>2</x:v>
       </x:c>
       <x:c r="F103" s="1" t="s">
-        <x:v>137</x:v>
+        <x:v>134</x:v>
       </x:c>
       <x:c r="G103" s="1" t="s">
         <x:v>50</x:v>
@@ -3597,19 +3585,19 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B104" s="8" t="s">
-        <x:v>209</x:v>
+        <x:v>205</x:v>
       </x:c>
       <x:c r="C104" s="9" t="s">
-        <x:v>210</x:v>
+        <x:v>206</x:v>
       </x:c>
       <x:c r="D104" s="8" t="s">
-        <x:v>211</x:v>
+        <x:v>207</x:v>
       </x:c>
       <x:c r="E104" s="8">
         <x:v>2</x:v>
       </x:c>
       <x:c r="F104" s="8" t="s">
-        <x:v>124</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="G104" s="8" t="s">
         <x:v>50</x:v>
@@ -3620,13 +3608,13 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B105" s="1" t="s">
-        <x:v>212</x:v>
+        <x:v>208</x:v>
       </x:c>
       <x:c r="C105" s="4" t="s">
-        <x:v>213</x:v>
+        <x:v>209</x:v>
       </x:c>
       <x:c r="D105" s="1" t="s">
-        <x:v>214</x:v>
+        <x:v>210</x:v>
       </x:c>
       <x:c r="E105" s="1">
         <x:v>1</x:v>
@@ -3643,19 +3631,19 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B106" s="8" t="s">
-        <x:v>212</x:v>
+        <x:v>208</x:v>
       </x:c>
       <x:c r="C106" s="9" t="s">
-        <x:v>213</x:v>
+        <x:v>209</x:v>
       </x:c>
       <x:c r="D106" s="8" t="s">
-        <x:v>215</x:v>
+        <x:v>211</x:v>
       </x:c>
       <x:c r="E106" s="8">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F106" s="8" t="s">
-        <x:v>137</x:v>
+        <x:v>134</x:v>
       </x:c>
       <x:c r="G106" s="8" t="s">
         <x:v>14</x:v>
@@ -3666,13 +3654,13 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B107" s="1" t="s">
-        <x:v>216</x:v>
+        <x:v>212</x:v>
       </x:c>
       <x:c r="C107" s="4" t="s">
-        <x:v>217</x:v>
+        <x:v>213</x:v>
       </x:c>
       <x:c r="D107" s="1" t="s">
-        <x:v>218</x:v>
+        <x:v>214</x:v>
       </x:c>
       <x:c r="E107" s="1">
         <x:v>2</x:v>
@@ -3689,19 +3677,19 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B108" s="8" t="s">
-        <x:v>219</x:v>
+        <x:v>215</x:v>
       </x:c>
       <x:c r="C108" s="9" t="s">
-        <x:v>220</x:v>
+        <x:v>216</x:v>
       </x:c>
       <x:c r="D108" s="8" t="s">
-        <x:v>221</x:v>
+        <x:v>217</x:v>
       </x:c>
       <x:c r="E108" s="8">
         <x:v>2</x:v>
       </x:c>
       <x:c r="F108" s="8" t="s">
-        <x:v>178</x:v>
+        <x:v>175</x:v>
       </x:c>
       <x:c r="G108" s="8" t="s">
         <x:v>50</x:v>
@@ -3712,13 +3700,13 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B109" s="1" t="s">
-        <x:v>222</x:v>
+        <x:v>218</x:v>
       </x:c>
       <x:c r="C109" s="4" t="s">
-        <x:v>223</x:v>
+        <x:v>219</x:v>
       </x:c>
       <x:c r="D109" s="1" t="s">
-        <x:v>224</x:v>
+        <x:v>220</x:v>
       </x:c>
       <x:c r="E109" s="1">
         <x:v>1</x:v>
@@ -3735,13 +3723,13 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B110" s="8" t="s">
+        <x:v>218</x:v>
+      </x:c>
+      <x:c r="C110" s="9" t="s">
+        <x:v>221</x:v>
+      </x:c>
+      <x:c r="D110" s="8" t="s">
         <x:v>222</x:v>
-      </x:c>
-      <x:c r="C110" s="9" t="s">
-        <x:v>225</x:v>
-      </x:c>
-      <x:c r="D110" s="8" t="s">
-        <x:v>226</x:v>
       </x:c>
       <x:c r="E110" s="8">
         <x:v>2</x:v>
@@ -3758,13 +3746,13 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B111" s="1" t="s">
-        <x:v>222</x:v>
+        <x:v>218</x:v>
       </x:c>
       <x:c r="C111" s="4" t="s">
-        <x:v>227</x:v>
+        <x:v>223</x:v>
       </x:c>
       <x:c r="D111" s="1" t="s">
-        <x:v>228</x:v>
+        <x:v>224</x:v>
       </x:c>
       <x:c r="E111" s="1">
         <x:v>2</x:v>
@@ -3781,13 +3769,13 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B112" s="8" t="s">
-        <x:v>222</x:v>
+        <x:v>218</x:v>
       </x:c>
       <x:c r="C112" s="9" t="s">
+        <x:v>221</x:v>
+      </x:c>
+      <x:c r="D112" s="8" t="s">
         <x:v>225</x:v>
-      </x:c>
-      <x:c r="D112" s="8" t="s">
-        <x:v>229</x:v>
       </x:c>
       <x:c r="E112" s="8">
         <x:v>1</x:v>
@@ -3804,13 +3792,13 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B113" s="1" t="s">
-        <x:v>222</x:v>
+        <x:v>218</x:v>
       </x:c>
       <x:c r="C113" s="4" t="s">
-        <x:v>223</x:v>
+        <x:v>219</x:v>
       </x:c>
       <x:c r="D113" s="1" t="s">
-        <x:v>230</x:v>
+        <x:v>226</x:v>
       </x:c>
       <x:c r="E113" s="1">
         <x:v>1</x:v>
@@ -3827,13 +3815,13 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B114" s="8" t="s">
-        <x:v>222</x:v>
+        <x:v>218</x:v>
       </x:c>
       <x:c r="C114" s="9" t="s">
-        <x:v>225</x:v>
+        <x:v>221</x:v>
       </x:c>
       <x:c r="D114" s="8" t="s">
-        <x:v>231</x:v>
+        <x:v>227</x:v>
       </x:c>
       <x:c r="E114" s="8">
         <x:v>1</x:v>
@@ -3850,13 +3838,13 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B115" s="1" t="s">
-        <x:v>222</x:v>
+        <x:v>218</x:v>
       </x:c>
       <x:c r="C115" s="4" t="s">
-        <x:v>225</x:v>
+        <x:v>221</x:v>
       </x:c>
       <x:c r="D115" s="1" t="s">
-        <x:v>232</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="E115" s="1">
         <x:v>1</x:v>
@@ -3873,13 +3861,13 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B116" s="8" t="s">
-        <x:v>222</x:v>
+        <x:v>218</x:v>
       </x:c>
       <x:c r="C116" s="9" t="s">
-        <x:v>233</x:v>
+        <x:v>229</x:v>
       </x:c>
       <x:c r="D116" s="8" t="s">
-        <x:v>234</x:v>
+        <x:v>230</x:v>
       </x:c>
       <x:c r="E116" s="8">
         <x:v>1</x:v>
@@ -3896,13 +3884,13 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B117" s="1" t="s">
-        <x:v>222</x:v>
+        <x:v>218</x:v>
       </x:c>
       <x:c r="C117" s="4" t="s">
-        <x:v>225</x:v>
+        <x:v>221</x:v>
       </x:c>
       <x:c r="D117" s="1" t="s">
-        <x:v>235</x:v>
+        <x:v>231</x:v>
       </x:c>
       <x:c r="E117" s="1">
         <x:v>1</x:v>
@@ -3919,19 +3907,19 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B118" s="8" t="s">
-        <x:v>222</x:v>
+        <x:v>218</x:v>
       </x:c>
       <x:c r="C118" s="9" t="s">
-        <x:v>223</x:v>
+        <x:v>219</x:v>
       </x:c>
       <x:c r="D118" s="8" t="s">
-        <x:v>236</x:v>
+        <x:v>232</x:v>
       </x:c>
       <x:c r="E118" s="8">
         <x:v>2</x:v>
       </x:c>
       <x:c r="F118" s="8" t="s">
-        <x:v>237</x:v>
+        <x:v>233</x:v>
       </x:c>
       <x:c r="G118" s="8" t="s">
         <x:v>58</x:v>
@@ -3942,13 +3930,13 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B119" s="1" t="s">
-        <x:v>222</x:v>
+        <x:v>218</x:v>
       </x:c>
       <x:c r="C119" s="4" t="s">
-        <x:v>225</x:v>
+        <x:v>221</x:v>
       </x:c>
       <x:c r="D119" s="1" t="s">
-        <x:v>238</x:v>
+        <x:v>234</x:v>
       </x:c>
       <x:c r="E119" s="1">
         <x:v>2</x:v>
@@ -3965,22 +3953,22 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B120" s="8" t="s">
+        <x:v>235</x:v>
+      </x:c>
+      <x:c r="C120" s="9" t="s">
+        <x:v>236</x:v>
+      </x:c>
+      <x:c r="D120" s="8" t="s">
+        <x:v>237</x:v>
+      </x:c>
+      <x:c r="E120" s="8">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F120" s="8" t="s">
+        <x:v>238</x:v>
+      </x:c>
+      <x:c r="G120" s="8" t="s">
         <x:v>239</x:v>
-      </x:c>
-      <x:c r="C120" s="9" t="s">
-        <x:v>240</x:v>
-      </x:c>
-      <x:c r="D120" s="8" t="s">
-        <x:v>241</x:v>
-      </x:c>
-      <x:c r="E120" s="8">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F120" s="8" t="s">
-        <x:v>242</x:v>
-      </x:c>
-      <x:c r="G120" s="8" t="s">
-        <x:v>243</x:v>
       </x:c>
     </x:row>
     <x:row r="121">
@@ -3988,22 +3976,22 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B121" s="1" t="s">
+        <x:v>235</x:v>
+      </x:c>
+      <x:c r="C121" s="4" t="s">
+        <x:v>236</x:v>
+      </x:c>
+      <x:c r="D121" s="1" t="s">
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="E121" s="1">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F121" s="1" t="s">
+        <x:v>238</x:v>
+      </x:c>
+      <x:c r="G121" s="1" t="s">
         <x:v>239</x:v>
-      </x:c>
-      <x:c r="C121" s="4" t="s">
-        <x:v>240</x:v>
-      </x:c>
-      <x:c r="D121" s="1" t="s">
-        <x:v>244</x:v>
-      </x:c>
-      <x:c r="E121" s="1">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F121" s="1" t="s">
-        <x:v>242</x:v>
-      </x:c>
-      <x:c r="G121" s="1" t="s">
-        <x:v>243</x:v>
       </x:c>
     </x:row>
     <x:row r="122">
@@ -4014,16 +4002,16 @@
         <x:v>0.56944444444444442</x:v>
       </x:c>
       <x:c r="C122" s="9" t="s">
-        <x:v>202</x:v>
+        <x:v>198</x:v>
       </x:c>
       <x:c r="D122" s="8" t="s">
-        <x:v>245</x:v>
+        <x:v>241</x:v>
       </x:c>
       <x:c r="E122" s="8">
         <x:v>2</x:v>
       </x:c>
       <x:c r="F122" s="8" t="s">
-        <x:v>199</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="G122" s="8" t="s">
         <x:v>50</x:v>
@@ -4034,19 +4022,19 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B123" s="1" t="s">
-        <x:v>246</x:v>
+        <x:v>242</x:v>
       </x:c>
       <x:c r="C123" s="4" t="s">
-        <x:v>247</x:v>
+        <x:v>243</x:v>
       </x:c>
       <x:c r="D123" s="1" t="s">
-        <x:v>248</x:v>
+        <x:v>244</x:v>
       </x:c>
       <x:c r="E123" s="1">
         <x:v>2</x:v>
       </x:c>
       <x:c r="F123" s="1" t="s">
-        <x:v>242</x:v>
+        <x:v>238</x:v>
       </x:c>
       <x:c r="G123" s="1" t="s">
         <x:v>50</x:v>
@@ -4057,19 +4045,19 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B124" s="8" t="s">
-        <x:v>249</x:v>
+        <x:v>245</x:v>
       </x:c>
       <x:c r="C124" s="9" t="s">
-        <x:v>250</x:v>
+        <x:v>246</x:v>
       </x:c>
       <x:c r="D124" s="8" t="s">
-        <x:v>251</x:v>
+        <x:v>247</x:v>
       </x:c>
       <x:c r="E124" s="8">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F124" s="8" t="s">
-        <x:v>242</x:v>
+        <x:v>238</x:v>
       </x:c>
       <x:c r="G124" s="8" t="s">
         <x:v>50</x:v>
@@ -4080,22 +4068,22 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B125" s="1" t="s">
-        <x:v>252</x:v>
+        <x:v>248</x:v>
       </x:c>
       <x:c r="C125" s="4" t="s">
-        <x:v>253</x:v>
+        <x:v>249</x:v>
       </x:c>
       <x:c r="D125" s="1" t="s">
-        <x:v>254</x:v>
+        <x:v>250</x:v>
       </x:c>
       <x:c r="E125" s="1">
         <x:v>2</x:v>
       </x:c>
       <x:c r="F125" s="1" t="s">
-        <x:v>88</x:v>
+        <x:v>86</x:v>
       </x:c>
       <x:c r="G125" s="1" t="s">
-        <x:v>89</x:v>
+        <x:v>87</x:v>
       </x:c>
     </x:row>
     <x:row r="126">
@@ -4103,22 +4091,22 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B126" s="8" t="s">
+        <x:v>248</x:v>
+      </x:c>
+      <x:c r="C126" s="9" t="s">
+        <x:v>251</x:v>
+      </x:c>
+      <x:c r="D126" s="8" t="s">
         <x:v>252</x:v>
       </x:c>
-      <x:c r="C126" s="9" t="s">
-        <x:v>255</x:v>
-      </x:c>
-      <x:c r="D126" s="8" t="s">
-        <x:v>256</x:v>
-      </x:c>
       <x:c r="E126" s="8">
         <x:v>2</x:v>
       </x:c>
       <x:c r="F126" s="8" t="s">
-        <x:v>257</x:v>
+        <x:v>253</x:v>
       </x:c>
       <x:c r="G126" s="8" t="s">
-        <x:v>89</x:v>
+        <x:v>87</x:v>
       </x:c>
     </x:row>
     <x:row r="127">
@@ -4126,22 +4114,22 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B127" s="1" t="s">
-        <x:v>252</x:v>
+        <x:v>248</x:v>
       </x:c>
       <x:c r="C127" s="4" t="s">
-        <x:v>258</x:v>
+        <x:v>254</x:v>
       </x:c>
       <x:c r="D127" s="1" t="s">
-        <x:v>259</x:v>
+        <x:v>255</x:v>
       </x:c>
       <x:c r="E127" s="1">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F127" s="1" t="s">
-        <x:v>257</x:v>
+        <x:v>253</x:v>
       </x:c>
       <x:c r="G127" s="1" t="s">
-        <x:v>89</x:v>
+        <x:v>87</x:v>
       </x:c>
     </x:row>
     <x:row r="128">
@@ -4149,22 +4137,22 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B128" s="8" t="s">
-        <x:v>252</x:v>
+        <x:v>248</x:v>
       </x:c>
       <x:c r="C128" s="9" t="s">
-        <x:v>260</x:v>
+        <x:v>256</x:v>
       </x:c>
       <x:c r="D128" s="8" t="s">
-        <x:v>261</x:v>
+        <x:v>257</x:v>
       </x:c>
       <x:c r="E128" s="8">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F128" s="8" t="s">
-        <x:v>257</x:v>
+        <x:v>253</x:v>
       </x:c>
       <x:c r="G128" s="8" t="s">
-        <x:v>89</x:v>
+        <x:v>87</x:v>
       </x:c>
     </x:row>
     <x:row r="129">
@@ -4172,22 +4160,22 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B129" s="1" t="s">
-        <x:v>252</x:v>
+        <x:v>248</x:v>
       </x:c>
       <x:c r="C129" s="4" t="s">
-        <x:v>262</x:v>
+        <x:v>258</x:v>
       </x:c>
       <x:c r="D129" s="1" t="s">
-        <x:v>263</x:v>
+        <x:v>259</x:v>
       </x:c>
       <x:c r="E129" s="1">
         <x:v>2</x:v>
       </x:c>
       <x:c r="F129" s="1" t="s">
-        <x:v>257</x:v>
+        <x:v>253</x:v>
       </x:c>
       <x:c r="G129" s="1" t="s">
-        <x:v>89</x:v>
+        <x:v>87</x:v>
       </x:c>
     </x:row>
     <x:row r="130">
@@ -4195,13 +4183,13 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B130" s="8" t="s">
-        <x:v>252</x:v>
+        <x:v>248</x:v>
       </x:c>
       <x:c r="C130" s="9" t="s">
-        <x:v>262</x:v>
+        <x:v>258</x:v>
       </x:c>
       <x:c r="D130" s="8" t="s">
-        <x:v>264</x:v>
+        <x:v>260</x:v>
       </x:c>
       <x:c r="E130" s="8">
         <x:v>1</x:v>
@@ -4210,7 +4198,7 @@
         <x:v>45</x:v>
       </x:c>
       <x:c r="G130" s="8" t="s">
-        <x:v>89</x:v>
+        <x:v>87</x:v>
       </x:c>
     </x:row>
     <x:row r="131">
@@ -4218,13 +4206,13 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B131" s="1" t="s">
-        <x:v>252</x:v>
+        <x:v>248</x:v>
       </x:c>
       <x:c r="C131" s="4" t="s">
-        <x:v>262</x:v>
+        <x:v>258</x:v>
       </x:c>
       <x:c r="D131" s="1" t="s">
-        <x:v>265</x:v>
+        <x:v>261</x:v>
       </x:c>
       <x:c r="E131" s="1">
         <x:v>1</x:v>
@@ -4233,7 +4221,7 @@
         <x:v>54</x:v>
       </x:c>
       <x:c r="G131" s="1" t="s">
-        <x:v>89</x:v>
+        <x:v>87</x:v>
       </x:c>
     </x:row>
     <x:row r="132">
@@ -4241,22 +4229,22 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B132" s="8" t="s">
-        <x:v>252</x:v>
+        <x:v>248</x:v>
       </x:c>
       <x:c r="C132" s="9" t="s">
-        <x:v>266</x:v>
+        <x:v>262</x:v>
       </x:c>
       <x:c r="D132" s="8" t="s">
-        <x:v>267</x:v>
+        <x:v>263</x:v>
       </x:c>
       <x:c r="E132" s="8">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F132" s="8" t="s">
-        <x:v>268</x:v>
+        <x:v>264</x:v>
       </x:c>
       <x:c r="G132" s="8" t="s">
-        <x:v>269</x:v>
+        <x:v>265</x:v>
       </x:c>
     </x:row>
     <x:row r="133">
@@ -4264,19 +4252,19 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B133" s="1" t="s">
-        <x:v>270</x:v>
+        <x:v>266</x:v>
       </x:c>
       <x:c r="C133" s="4" t="s">
-        <x:v>271</x:v>
+        <x:v>267</x:v>
       </x:c>
       <x:c r="D133" s="1" t="s">
-        <x:v>272</x:v>
+        <x:v>268</x:v>
       </x:c>
       <x:c r="E133" s="1">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F133" s="1" t="s">
-        <x:v>178</x:v>
+        <x:v>175</x:v>
       </x:c>
       <x:c r="G133" s="1" t="s">
         <x:v>14</x:v>
@@ -4293,7 +4281,7 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="D134" s="8" t="s">
-        <x:v>273</x:v>
+        <x:v>269</x:v>
       </x:c>
       <x:c r="E134" s="8">
         <x:v>2</x:v>
@@ -4313,10 +4301,10 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="C135" s="4" t="s">
-        <x:v>274</x:v>
+        <x:v>270</x:v>
       </x:c>
       <x:c r="D135" s="1" t="s">
-        <x:v>275</x:v>
+        <x:v>271</x:v>
       </x:c>
       <x:c r="E135" s="1">
         <x:v>1</x:v>
@@ -4333,22 +4321,22 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B136" s="8" t="s">
-        <x:v>276</x:v>
+        <x:v>272</x:v>
       </x:c>
       <x:c r="C136" s="9" t="s">
-        <x:v>277</x:v>
+        <x:v>273</x:v>
       </x:c>
       <x:c r="D136" s="8" t="s">
-        <x:v>278</x:v>
+        <x:v>274</x:v>
       </x:c>
       <x:c r="E136" s="8">
         <x:v>2</x:v>
       </x:c>
       <x:c r="F136" s="8" t="s">
-        <x:v>199</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="G136" s="8" t="s">
-        <x:v>279</x:v>
+        <x:v>275</x:v>
       </x:c>
     </x:row>
     <x:row r="137">
@@ -4356,13 +4344,13 @@
         <x:v>46330</x:v>
       </x:c>
       <x:c r="B137" s="1" t="s">
-        <x:v>280</x:v>
+        <x:v>276</x:v>
       </x:c>
       <x:c r="C137" s="4" t="s">
-        <x:v>281</x:v>
+        <x:v>277</x:v>
       </x:c>
       <x:c r="D137" s="1" t="s">
-        <x:v>282</x:v>
+        <x:v>278</x:v>
       </x:c>
       <x:c r="E137" s="1">
         <x:v>1</x:v>
@@ -4382,19 +4370,19 @@
         <x:v>7.2916666666666671E-2</x:v>
       </x:c>
       <x:c r="C138" s="9" t="s">
-        <x:v>283</x:v>
+        <x:v>279</x:v>
       </x:c>
       <x:c r="D138" s="8" t="s">
-        <x:v>284</x:v>
+        <x:v>280</x:v>
       </x:c>
       <x:c r="E138" s="8">
         <x:v>2</x:v>
       </x:c>
       <x:c r="F138" s="8" t="s">
-        <x:v>257</x:v>
+        <x:v>253</x:v>
       </x:c>
       <x:c r="G138" s="8" t="s">
-        <x:v>89</x:v>
+        <x:v>87</x:v>
       </x:c>
     </x:row>
     <x:row r="139">
@@ -4402,22 +4390,22 @@
         <x:v>46331</x:v>
       </x:c>
       <x:c r="B139" s="1" t="s">
-        <x:v>252</x:v>
+        <x:v>248</x:v>
       </x:c>
       <x:c r="C139" s="4" t="s">
-        <x:v>253</x:v>
+        <x:v>249</x:v>
       </x:c>
       <x:c r="D139" s="1" t="s">
-        <x:v>285</x:v>
+        <x:v>281</x:v>
       </x:c>
       <x:c r="E139" s="1">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F139" s="1" t="s">
-        <x:v>97</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="G139" s="1" t="s">
-        <x:v>89</x:v>
+        <x:v>87</x:v>
       </x:c>
     </x:row>
     <x:row r="140">
@@ -4425,22 +4413,22 @@
         <x:v>46331</x:v>
       </x:c>
       <x:c r="B140" s="8" t="s">
+        <x:v>282</x:v>
+      </x:c>
+      <x:c r="C140" s="9" t="s">
+        <x:v>283</x:v>
+      </x:c>
+      <x:c r="D140" s="8" t="s">
+        <x:v>284</x:v>
+      </x:c>
+      <x:c r="E140" s="8">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F140" s="8" t="s">
+        <x:v>285</x:v>
+      </x:c>
+      <x:c r="G140" s="8" t="s">
         <x:v>286</x:v>
-      </x:c>
-      <x:c r="C140" s="9" t="s">
-        <x:v>287</x:v>
-      </x:c>
-      <x:c r="D140" s="8" t="s">
-        <x:v>288</x:v>
-      </x:c>
-      <x:c r="E140" s="8">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="F140" s="8" t="s">
-        <x:v>289</x:v>
-      </x:c>
-      <x:c r="G140" s="8" t="s">
-        <x:v>290</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4457,21 +4445,21 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="10" t="s">
-        <x:v>291</x:v>
+        <x:v>287</x:v>
       </x:c>
       <x:c r="B1" s="10"/>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="11" t="s">
-        <x:v>292</x:v>
+        <x:v>288</x:v>
       </x:c>
       <x:c r="B2" s="11" t="s">
-        <x:v>293</x:v>
+        <x:v>289</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="1" t="s">
-        <x:v>294</x:v>
+        <x:v>290</x:v>
       </x:c>
       <x:c r="B3" s="3">
         <x:v>8.3333333333333329E-2</x:v>
@@ -4479,7 +4467,7 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="1" t="s">
-        <x:v>295</x:v>
+        <x:v>291</x:v>
       </x:c>
       <x:c r="B4" s="3">
         <x:v>0.125</x:v>
@@ -4487,7 +4475,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="1" t="s">
-        <x:v>296</x:v>
+        <x:v>292</x:v>
       </x:c>
       <x:c r="B5" s="3">
         <x:v>0.16666666666666666</x:v>
@@ -4495,7 +4483,7 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="1" t="s">
-        <x:v>297</x:v>
+        <x:v>293</x:v>
       </x:c>
       <x:c r="B6" s="3">
         <x:v>0.25</x:v>
@@ -4503,7 +4491,7 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="1" t="s">
-        <x:v>298</x:v>
+        <x:v>294</x:v>
       </x:c>
       <x:c r="B7" s="3">
         <x:v>0.33333333333333331</x:v>
@@ -4511,7 +4499,7 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="1" t="s">
-        <x:v>299</x:v>
+        <x:v>295</x:v>
       </x:c>
       <x:c r="B8" s="12">
         <x:v>0.41666666666666669</x:v>
@@ -4523,21 +4511,21 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="10" t="s">
-        <x:v>300</x:v>
+        <x:v>296</x:v>
       </x:c>
       <x:c r="B10" s="10"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="11" t="s">
-        <x:v>292</x:v>
+        <x:v>288</x:v>
       </x:c>
       <x:c r="B11" s="11" t="s">
-        <x:v>293</x:v>
+        <x:v>289</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="1" t="s">
-        <x:v>294</x:v>
+        <x:v>290</x:v>
       </x:c>
       <x:c r="B12" s="3">
         <x:v>8.3333333333333329E-2</x:v>
@@ -4545,7 +4533,7 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="1" t="s">
-        <x:v>295</x:v>
+        <x:v>291</x:v>
       </x:c>
       <x:c r="B13" s="3">
         <x:v>0.125</x:v>
@@ -4553,7 +4541,7 @@
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="1" t="s">
-        <x:v>296</x:v>
+        <x:v>292</x:v>
       </x:c>
       <x:c r="B14" s="3">
         <x:v>0.16666666666666666</x:v>
@@ -4561,7 +4549,7 @@
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="1" t="s">
-        <x:v>297</x:v>
+        <x:v>293</x:v>
       </x:c>
       <x:c r="B15" s="3">
         <x:v>0.25</x:v>
@@ -4569,7 +4557,7 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="1" t="s">
-        <x:v>298</x:v>
+        <x:v>294</x:v>
       </x:c>
       <x:c r="B16" s="3">
         <x:v>0.33333333333333331</x:v>
@@ -4577,7 +4565,7 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="1" t="s">
-        <x:v>299</x:v>
+        <x:v>295</x:v>
       </x:c>
       <x:c r="B17" s="12">
         <x:v>0.41666666666666669</x:v>
@@ -4589,21 +4577,21 @@
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="10" t="s">
-        <x:v>301</x:v>
+        <x:v>297</x:v>
       </x:c>
       <x:c r="B19" s="10"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="11" t="s">
-        <x:v>292</x:v>
+        <x:v>288</x:v>
       </x:c>
       <x:c r="B20" s="11" t="s">
-        <x:v>293</x:v>
+        <x:v>289</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="1" t="s">
-        <x:v>294</x:v>
+        <x:v>290</x:v>
       </x:c>
       <x:c r="B21" s="3">
         <x:v>8.3333333333333329E-2</x:v>
@@ -4611,7 +4599,7 @@
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="1" t="s">
-        <x:v>295</x:v>
+        <x:v>291</x:v>
       </x:c>
       <x:c r="B22" s="3">
         <x:v>0.125</x:v>
@@ -4619,7 +4607,7 @@
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="1" t="s">
-        <x:v>296</x:v>
+        <x:v>292</x:v>
       </x:c>
       <x:c r="B23" s="3">
         <x:v>0.16666666666666666</x:v>
@@ -4627,7 +4615,7 @@
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="1" t="s">
-        <x:v>297</x:v>
+        <x:v>293</x:v>
       </x:c>
       <x:c r="B24" s="3">
         <x:v>0.25</x:v>
@@ -4635,7 +4623,7 @@
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="1" t="s">
-        <x:v>298</x:v>
+        <x:v>294</x:v>
       </x:c>
       <x:c r="B25" s="3">
         <x:v>0.33333333333333331</x:v>
@@ -4643,7 +4631,7 @@
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="1" t="s">
-        <x:v>299</x:v>
+        <x:v>295</x:v>
       </x:c>
       <x:c r="B26" s="12">
         <x:v>0.41666666666666669</x:v>

</xml_diff>